<commit_message>
Add demo-data disclaimer to sample report and portfolio folder
</commit_message>
<xml_diff>
--- a/portfolio_sample/Ecommerce_Analytics_Report_SAMPLE.xlsx
+++ b/portfolio_sample/Ecommerce_Analytics_Report_SAMPLE.xlsx
@@ -7,19 +7,20 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sales_Trends_Daily" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sales_Trends_Monthly" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Customer_Behavior" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Product_Performance" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Category_Breakdown" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Read_Me_First" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sales_Trends_Daily" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sales_Trends_Monthly" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Customer_Behavior" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Product_Performance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Category_Breakdown" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sales_Trends_Daily'!$A$1:$C$91</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sales_Trends_Monthly'!$A$1:$C$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Customer_Behavior'!$A$1:$F$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Product_Performance'!$A$1:$D$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Category_Breakdown'!$A$1:$C$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sales_Trends_Daily'!$A$1:$C$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sales_Trends_Monthly'!$A$1:$C$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Customer_Behavior'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Product_Performance'!$A$1:$D$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Category_Breakdown'!$A$1:$C$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -31,7 +32,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +49,14 @@
     </font>
     <font>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -90,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -108,6 +117,8 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -742,6 +753,78 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="85" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>DEMO / SAMPLE REPORT — NOT REAL CLIENT DATA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>This report and the accompanying Orders_Sample.csv were generated from</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>synthetic, randomly created data (see make_sample_data.py) purely to</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>demonstrate how the Ecommerce Analytics Engine cleans data and builds</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>reports.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>It does not represent any real store, business, or client, and no actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>client data was used or shared in producing this sample.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -833,7 +916,6 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -880,7 +962,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1907,7 +1989,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1984,7 +2066,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2259,7 +2341,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2463,7 +2545,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>